<commit_message>
add verified software copyright record
</commit_message>
<xml_diff>
--- a/frontend/data-source/software-copyrights.xlsx
+++ b/frontend/data-source/software-copyrights.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="软件著作" sheetId="1" r:id="R31e14ffa95154809"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="软件著作" sheetId="1" r:id="R8fe53c73e7f04f54"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +13,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="3">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="0"/>
+  </x:numFmts>
+  <x:fonts count="4">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -28,6 +31,11 @@
       <x:b/>
       <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF2B2430"/>
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
@@ -50,7 +58,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="6">
+  <x:cellXfs count="10">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -62,6 +70,18 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -265,12 +285,12 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="56" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="44" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="58" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="76" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="27" customHeight="1">
@@ -293,6 +313,26 @@
         <x:v>note</x:v>
       </x:c>
     </x:row>
+    <x:row r="2" ht="74" customHeight="1">
+      <x:c r="A2" s="8" t="str">
+        <x:v>software-001</x:v>
+      </x:c>
+      <x:c r="B2" s="8" t="str">
+        <x:v>标准驱动的集成化众测服务平台V3.0</x:v>
+      </x:c>
+      <x:c r="C2" s="8" t="str">
+        <x:v>2022SR0042472</x:v>
+      </x:c>
+      <x:c r="D2" s="9" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="E2" s="8" t="str">
+        <x:v>广东拓思软件科学园有限公司;南京慕测信息科技有限公司;上海计算机软件技术开发中心;航天中认软件测评科技(北京)有限责任公司</x:v>
+      </x:c>
+      <x:c r="F2" s="8" t="str">
+        <x:v>来源：2023年度广东省科技进步奖提名项目公示（成果与陈振宇、房春荣参与的“群智驱动众测关键技术研究及其应用”项目关联）：https://www.gdktzx.com/d/file/2023/12/b63ec1e9c01d4dc001e786a6ffe777a0.pdf</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>